<commit_message>
feat(site): update leaderboard data and mobile headings
</commit_message>
<xml_diff>
--- a/料力榜.xlsx
+++ b/料力榜.xlsx
@@ -16,6 +16,9 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$B$2:$K$13</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -34,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="59">
   <si>
     <t>日期</t>
   </si>
@@ -72,7 +75,7 @@
     <t>加点滋味</t>
   </si>
   <si>
-    <t>肉蟹煲</t>
+    <t>肉蟹煲料包</t>
   </si>
   <si>
     <t>鲜香微辣，值得一试</t>
@@ -99,7 +102,7 @@
     <t>EP3</t>
   </si>
   <si>
-    <t>芥末小海鲜</t>
+    <t>芥末小海鲜捞汁</t>
   </si>
   <si>
     <t>芥味清爽，略欠鲜香</t>
@@ -111,7 +114,7 @@
     <t>EP4</t>
   </si>
   <si>
-    <t>云南油焖鸡</t>
+    <t>云南油焖鸡料包</t>
   </si>
   <si>
     <t>辣而少香，入味欠佳</t>
@@ -150,7 +153,7 @@
     <t>EP7</t>
   </si>
   <si>
-    <t>牛肉麻婆豆腐</t>
+    <t>牛肉麻婆豆腐料包</t>
   </si>
   <si>
     <t>咸重压味，麻香不足</t>
@@ -165,7 +168,7 @@
     <t>山姆</t>
   </si>
   <si>
-    <t>金汤肥牛</t>
+    <t>金汤肥牛调味料</t>
   </si>
   <si>
     <t>酸辣突出，香味稍弱</t>
@@ -192,7 +195,25 @@
     <t>EP10</t>
   </si>
   <si>
+    <t>沃集鲜</t>
+  </si>
+  <si>
+    <t>党参黄芪骨汤米线</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>药香突出，鸡肉提鲜</t>
+  </si>
+  <si>
     <t>EP11</t>
+  </si>
+  <si>
+    <t>海南鸡饭煮饭料</t>
+  </si>
+  <si>
+    <t>米香油润，鸡鲜味足</t>
   </si>
 </sst>
 </file>
@@ -1205,7 +1226,7 @@
   <cols>
     <col min="2" max="2" width="13.0176991150442" customWidth="1"/>
     <col min="4" max="4" width="10.8318584070796" style="1" customWidth="1"/>
-    <col min="5" max="5" width="15.7699115044248" style="1" customWidth="1"/>
+    <col min="5" max="5" width="19.0619469026549" style="1" customWidth="1"/>
     <col min="6" max="8" width="9" style="1"/>
     <col min="9" max="9" width="12.7964601769912" style="1"/>
     <col min="10" max="10" width="21.5752212389381" customWidth="1"/>
@@ -1541,41 +1562,65 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1" spans="2:11">
-      <c r="B12" s="8">
-        <v>46298</v>
-      </c>
-      <c r="C12" s="9" t="s">
+      <c r="B12" s="4">
+        <v>46305</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="D12" s="9"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="11" t="e">
+      <c r="D12" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F12" s="5">
+        <v>3.9</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="H12" s="5">
+        <v>4.3</v>
+      </c>
+      <c r="I12" s="7">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J12" s="11"/>
-      <c r="K12" s="12"/>
+        <v>4.1</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="K12" s="7"/>
     </row>
     <row r="13" ht="20" customHeight="1" spans="2:11">
       <c r="B13" s="8">
-        <v>46302</v>
+        <v>46308</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="D13" s="9"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="11" t="e">
+        <v>56</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="F13" s="11">
+        <v>4.2</v>
+      </c>
+      <c r="G13" s="9">
+        <v>4</v>
+      </c>
+      <c r="H13" s="9">
+        <v>4.3</v>
+      </c>
+      <c r="I13" s="11">
         <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="J13" s="11"/>
+        <v>4.16666666666667</v>
+      </c>
+      <c r="J13" s="11" t="s">
+        <v>58</v>
+      </c>
       <c r="K13" s="12"/>
     </row>
     <row r="14" ht="20" customHeight="1"/>
@@ -1585,6 +1630,9 @@
     <row r="18" ht="20" customHeight="1"/>
     <row r="19" ht="20" customHeight="1"/>
   </sheetData>
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="B2:K13" etc:filterBottomFollowUsedRange="0">
+    <extLst/>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter/>

</xml_diff>